<commit_message>
Daily NSE scan: 2026-09-03
</commit_message>
<xml_diff>
--- a/output/2026-09-03/enriched_analysis.xlsx
+++ b/output/2026-09-03/enriched_analysis.xlsx
@@ -1390,7 +1390,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1609,27 +1609,27 @@
         <v>109.51</v>
       </c>
       <c r="J12" t="n">
-        <v>91.62</v>
+        <v>91.7</v>
       </c>
       <c r="K12" t="n">
-        <v>19.5</v>
+        <v>19.4</v>
       </c>
       <c r="L12" t="n">
         <v>70.88</v>
       </c>
       <c r="M12" t="n">
-        <v>8.390000000000001</v>
+        <v>8.49</v>
       </c>
       <c r="N12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>01-09-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.298</v>
+        <v>0.302</v>
       </c>
       <c r="Q12" t="n">
         <v>2815</v>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ganesh Consumer Products Limited</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -5400,7 +5400,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5477,23 +5477,23 @@
         <v>109.51</v>
       </c>
       <c r="D12" t="n">
-        <v>91.62</v>
+        <v>91.7</v>
       </c>
       <c r="E12" t="n">
-        <v>19.5</v>
+        <v>19.4</v>
       </c>
       <c r="F12" t="n">
         <v>70.88</v>
       </c>
       <c r="G12" t="n">
-        <v>8.390000000000001</v>
+        <v>8.49</v>
       </c>
       <c r="H12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>01-09-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
     </row>
@@ -6170,7 +6170,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ganesh Consumer Products Limited</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C32" t="n">

</xml_diff>